<commit_message>
refactor: update Employee component styles and improve UI consistency
- Refactored button styles in Employee component for better visual consistency and accessibility.
- Updated CSS variables for a light theme palette, enhancing readability and aesthetics.
- Introduced Tailwind CSS configuration for streamlined styling across the application.
- Adjusted background and text colors to align with the new design guidelines.
</commit_message>
<xml_diff>
--- a/data/employee-management.xlsx
+++ b/data/employee-management.xlsx
@@ -1162,7 +1162,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:J5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1172,24 +1172,27 @@
         <v>EmployeeID</v>
       </c>
       <c r="C1" t="str">
+        <v>CompanyID</v>
+      </c>
+      <c r="D1" t="str">
         <v>WorkTitle</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>StartDate</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>EndDate</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>WorkAmount</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>ReceivedAmount</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>PendingAmount</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Status</v>
       </c>
     </row>
@@ -1201,24 +1204,27 @@
         <v>EMP002</v>
       </c>
       <c r="C2" t="str">
+        <v>CMP002</v>
+      </c>
+      <c r="D2" t="str">
         <v>Kiln lining repair</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>2026-05-01</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>2026-05-12</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <v>28000</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>10000</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>18000</v>
       </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
         <v>Ongoing</v>
       </c>
     </row>
@@ -1230,24 +1236,27 @@
         <v>EMP003</v>
       </c>
       <c r="C3" t="str">
+        <v>CMP001</v>
+      </c>
+      <c r="D3" t="str">
         <v>Dispatch bay rework</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F3" t="str">
         <v>2026-05-06</v>
-      </c>
-      <c r="F3">
-        <v>18000</v>
       </c>
       <c r="G3">
         <v>18000</v>
       </c>
       <c r="H3">
+        <v>18000</v>
+      </c>
+      <c r="I3">
         <v>0</v>
       </c>
-      <c r="I3" t="str">
+      <c r="J3" t="str">
         <v>Completed</v>
       </c>
     </row>
@@ -1259,24 +1268,27 @@
         <v>EMP001</v>
       </c>
       <c r="C4" t="str">
+        <v>CMP001</v>
+      </c>
+      <c r="D4" t="str">
         <v>Raw mix inspection</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
         <v>2026-05-03</v>
       </c>
-      <c r="E4" t="str">
+      <c r="F4" t="str">
         <v>2026-05-16</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <v>14500</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>7000</v>
       </c>
-      <c r="H4">
+      <c r="I4">
         <v>7500</v>
       </c>
-      <c r="I4" t="str">
+      <c r="J4" t="str">
         <v>Ongoing</v>
       </c>
     </row>
@@ -1288,30 +1300,33 @@
         <v>EMP004</v>
       </c>
       <c r="C5" t="str">
+        <v>CMP001</v>
+      </c>
+      <c r="D5" t="str">
         <v>Warehouse inventory audit</v>
       </c>
-      <c r="D5" t="str">
+      <c r="E5" t="str">
         <v>2026-04-20</v>
       </c>
-      <c r="E5" t="str">
+      <c r="F5" t="str">
         <v>2026-05-02</v>
-      </c>
-      <c r="F5">
-        <v>12250</v>
       </c>
       <c r="G5">
         <v>12250</v>
       </c>
       <c r="H5">
+        <v>12250</v>
+      </c>
+      <c r="I5">
         <v>0</v>
       </c>
-      <c r="I5" t="str">
+      <c r="J5" t="str">
         <v>Completed</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>